<commit_message>
Daily NSE scan: 2026-09-28
</commit_message>
<xml_diff>
--- a/output/2026-09-28/enriched_analysis.xlsx
+++ b/output/2026-09-28/enriched_analysis.xlsx
@@ -929,10 +929,10 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>3.274</v>
+        <v>3.279</v>
       </c>
       <c r="W2" t="n">
-        <v>2933</v>
+        <v>2928</v>
       </c>
       <c r="X2" t="n">
         <v>23</v>
@@ -1161,13 +1161,13 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>0.844</v>
+        <v>0.826</v>
       </c>
       <c r="W3" t="n">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="X3" t="n">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="Y3" t="n">
         <v>22</v>
@@ -1393,10 +1393,10 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>0.928</v>
+        <v>0.952</v>
       </c>
       <c r="W4" t="n">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="n">
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1568,7 +1568,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F5" t="n">
         <v>19</v>
@@ -1623,13 +1623,13 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>1.003</v>
+        <v>0.974</v>
       </c>
       <c r="W5" t="n">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="X5" t="n">
-        <v>8.51</v>
+        <v>8.73</v>
       </c>
       <c r="Y5" t="n">
         <v>17</v>
@@ -1858,10 +1858,10 @@
         <v>0.052</v>
       </c>
       <c r="W6" t="n">
-        <v>2561</v>
+        <v>2556</v>
       </c>
       <c r="X6" t="n">
-        <v>8.800000000000001</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="Y6" t="n">
         <v>36</v>
@@ -2087,13 +2087,13 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>0.445</v>
+        <v>0.443</v>
       </c>
       <c r="W7" t="n">
-        <v>2736</v>
+        <v>2748</v>
       </c>
       <c r="X7" t="n">
-        <v>22.4</v>
+        <v>22.5</v>
       </c>
       <c r="Y7" t="n">
         <v>8</v>
@@ -2319,13 +2319,13 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>0.121</v>
+        <v>0.12</v>
       </c>
       <c r="W8" t="n">
-        <v>2594</v>
+        <v>2624</v>
       </c>
       <c r="X8" t="n">
-        <v>22.7</v>
+        <v>23</v>
       </c>
       <c r="Y8" t="n">
         <v>-3</v>
@@ -2551,13 +2551,13 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>0.3</v>
+        <v>0.307</v>
       </c>
       <c r="W9" t="n">
-        <v>1021</v>
+        <v>999</v>
       </c>
       <c r="X9" t="n">
-        <v>10</v>
+        <v>9.82</v>
       </c>
       <c r="Y9" t="n">
         <v>7</v>
@@ -2783,13 +2783,13 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>0.048</v>
+        <v>0.05</v>
       </c>
       <c r="W10" t="n">
-        <v>1722</v>
+        <v>1637</v>
       </c>
       <c r="X10" t="n">
-        <v>23.2</v>
+        <v>22</v>
       </c>
       <c r="Y10" t="n">
         <v>55</v>
@@ -3015,10 +3015,10 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>1.814</v>
+        <v>1.785</v>
       </c>
       <c r="W11" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="n">
@@ -3245,13 +3245,13 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>0.045</v>
+        <v>0.046</v>
       </c>
       <c r="W12" t="n">
-        <v>15959</v>
+        <v>15696</v>
       </c>
       <c r="X12" t="n">
-        <v>40.6</v>
+        <v>40</v>
       </c>
       <c r="Y12" t="n">
         <v>83</v>
@@ -3477,13 +3477,13 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>0.143</v>
+        <v>0.13</v>
       </c>
       <c r="W13" t="n">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="X13" t="n">
-        <v>32.6</v>
+        <v>35.9</v>
       </c>
       <c r="Y13" t="n">
         <v>19</v>
@@ -3709,13 +3709,13 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>2.29</v>
+        <v>2.324</v>
       </c>
       <c r="W14" t="n">
-        <v>2563</v>
+        <v>2526</v>
       </c>
       <c r="X14" t="n">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="Y14" t="n">
         <v>6</v>
@@ -3869,12 +3869,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>STEL HOLDINGS LIMITED</t>
+          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -3886,40 +3886,40 @@
         </is>
       </c>
       <c r="E15" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" t="n">
         <v>12</v>
       </c>
-      <c r="F15" t="n">
-        <v>13</v>
-      </c>
       <c r="G15" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H15" t="n">
         <v>-1</v>
       </c>
       <c r="I15" t="n">
-        <v>619.3</v>
+        <v>191.99</v>
       </c>
       <c r="J15" t="n">
-        <v>636.71</v>
+        <v>170.45</v>
       </c>
       <c r="K15" t="n">
-        <v>-2.7</v>
+        <v>12.6</v>
       </c>
       <c r="L15" t="n">
-        <v>64.68000000000001</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="M15" t="n">
-        <v>4.12</v>
+        <v>0.26</v>
       </c>
       <c r="N15" t="n">
-        <v>41238002</v>
+        <v>2560187</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>41238002</v>
+        <v>2560187</v>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
@@ -3933,64 +3933,64 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="V15" t="n">
-        <v>0.361</v>
+        <v>0.1</v>
       </c>
       <c r="W15" t="n">
-        <v>1143</v>
+        <v>256</v>
       </c>
       <c r="X15" t="n">
-        <v>58.2</v>
+        <v>27.4</v>
       </c>
       <c r="Y15" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="Z15" t="n">
-        <v>-0.11</v>
+        <v>1.87</v>
       </c>
       <c r="AA15" t="n">
-        <v>23</v>
+        <v>-31</v>
       </c>
       <c r="AB15" t="n">
-        <v>-0.07000000000000001</v>
+        <v>3.36</v>
       </c>
       <c r="AC15" t="n">
-        <v>1.58</v>
+        <v>4.96</v>
       </c>
       <c r="AD15" t="n">
         <v>0</v>
       </c>
       <c r="AE15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF15" t="n">
-        <v>-110</v>
+        <v>2.97</v>
       </c>
       <c r="AG15" t="n">
-        <v>590.22</v>
+        <v>181.14</v>
       </c>
       <c r="AH15" t="n">
-        <v>518.25</v>
+        <v>163.73</v>
       </c>
       <c r="AI15" t="n">
-        <v>45.3</v>
+        <v>57.4</v>
       </c>
       <c r="AJ15" t="n">
-        <v>636.7131718313339</v>
+        <v>170.4518641810919</v>
       </c>
       <c r="AK15" t="n">
-        <v>-2.7</v>
+        <v>12.6</v>
       </c>
       <c r="AL15" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="AM15" t="inlineStr">
@@ -4000,57 +4000,57 @@
       </c>
       <c r="AN15" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AO15" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="AQ15" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="AR15" t="n">
-        <v>95</v>
+        <v>25</v>
       </c>
       <c r="AS15" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="AT15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AU15" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AV15" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="AW15" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="AX15" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="AY15" t="n">
-        <v>2255167</v>
+        <v>0</v>
       </c>
       <c r="AZ15" t="n">
-        <v>16560542</v>
+        <v>0</v>
       </c>
       <c r="BA15" t="n">
-        <v>21276462</v>
+        <v>2560187</v>
       </c>
       <c r="BB15" t="n">
-        <v>38328962</v>
+        <v>2560187</v>
       </c>
       <c r="BC15" t="n">
-        <v>38328962</v>
+        <v>2560187</v>
       </c>
       <c r="BD15" t="n">
         <v>0</v>
@@ -4083,10 +4083,10 @@
         <v>0</v>
       </c>
       <c r="BN15" t="n">
-        <v>2255167</v>
+        <v>0</v>
       </c>
       <c r="BO15" t="n">
-        <v>21276462</v>
+        <v>2560187</v>
       </c>
       <c r="BP15" t="n">
         <v>2</v>
@@ -4095,22 +4095,22 @@
         <v>0</v>
       </c>
       <c r="BR15" t="n">
-        <v>0.106</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ASAHISONG</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ASAHI SONGWON COLORS LIMITED</t>
+          <t>STEL HOLDINGS LIMITED</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -4118,171 +4118,171 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F16" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G16" t="n">
+        <v>17</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I16" t="n">
+        <v>619.3</v>
+      </c>
+      <c r="J16" t="n">
+        <v>636.71</v>
+      </c>
+      <c r="K16" t="n">
+        <v>-2.7</v>
+      </c>
+      <c r="L16" t="n">
+        <v>64.68000000000001</v>
+      </c>
+      <c r="M16" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="N16" t="n">
+        <v>41238002</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>41238002</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Net Buying</t>
+        </is>
+      </c>
+      <c r="S16" t="b">
+        <v>0</v>
+      </c>
+      <c r="T16" t="n">
+        <v>34</v>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>24-09-2026</t>
+        </is>
+      </c>
+      <c r="V16" t="n">
+        <v>0.356</v>
+      </c>
+      <c r="W16" t="n">
+        <v>1160</v>
+      </c>
+      <c r="X16" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="Y16" t="n">
         <v>21</v>
       </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>402.75</v>
-      </c>
-      <c r="J16" t="n">
-        <v>338.1</v>
-      </c>
-      <c r="K16" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="L16" t="n">
-        <v>66.73</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="N16" t="n">
-        <v>3381000</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="n">
-        <v>3381000</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>Net Buying</t>
-        </is>
-      </c>
-      <c r="S16" t="b">
-        <v>0</v>
-      </c>
-      <c r="T16" t="n">
-        <v>1</v>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>11-08-2026</t>
-        </is>
-      </c>
-      <c r="V16" t="n">
-        <v>0.07099999999999999</v>
-      </c>
-      <c r="W16" t="n">
-        <v>475</v>
-      </c>
-      <c r="X16" t="n">
+      <c r="Z16" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>23</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>-110</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>590.22</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>518.25</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>636.7131718313339</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>-2.7</v>
+      </c>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>Fresh</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>24-09-2026</t>
+        </is>
+      </c>
+      <c r="AQ16" t="n">
+        <v>91</v>
+      </c>
+      <c r="AR16" t="n">
+        <v>95</v>
+      </c>
+      <c r="AS16" t="n">
+        <v>4</v>
+      </c>
+      <c r="AT16" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU16" t="n">
+        <v>8</v>
+      </c>
+      <c r="AV16" t="n">
         <v>14</v>
       </c>
-      <c r="Y16" t="n">
-        <v>-8</v>
-      </c>
-      <c r="Z16" t="n">
-        <v>24</v>
-      </c>
-      <c r="AA16" t="n">
+      <c r="AW16" t="n">
         <v>33</v>
       </c>
-      <c r="AB16" t="n">
-        <v>14.36</v>
-      </c>
-      <c r="AC16" t="n">
-        <v>9.94</v>
-      </c>
-      <c r="AD16" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="AE16" t="b">
-        <v>1</v>
-      </c>
-      <c r="AF16" t="n">
-        <v>18</v>
-      </c>
-      <c r="AG16" t="n">
-        <v>359.64</v>
-      </c>
-      <c r="AH16" t="n">
-        <v>270.07</v>
-      </c>
-      <c r="AI16" t="n">
-        <v>101.1</v>
-      </c>
-      <c r="AJ16" t="n">
-        <v>338.1</v>
-      </c>
-      <c r="AK16" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="AL16" t="inlineStr">
-        <is>
-          <t>Aging</t>
-        </is>
-      </c>
-      <c r="AM16" t="inlineStr">
-        <is>
-          <t>Mature Accumulation</t>
-        </is>
-      </c>
-      <c r="AN16" t="inlineStr">
-        <is>
-          <t>Mature — Wait for Pullback</t>
-        </is>
-      </c>
-      <c r="AO16" t="inlineStr">
-        <is>
-          <t>11-08-2026</t>
-        </is>
-      </c>
-      <c r="AP16" t="inlineStr">
-        <is>
-          <t>11-08-2026</t>
-        </is>
-      </c>
-      <c r="AQ16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR16" t="n">
-        <v>48</v>
-      </c>
-      <c r="AS16" t="n">
-        <v>48</v>
-      </c>
-      <c r="AT16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW16" t="n">
-        <v>1</v>
-      </c>
       <c r="AX16" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="AY16" t="n">
-        <v>0</v>
+        <v>2255167</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0</v>
+        <v>16560542</v>
       </c>
       <c r="BA16" t="n">
-        <v>0</v>
+        <v>21276462</v>
       </c>
       <c r="BB16" t="n">
-        <v>3381000</v>
+        <v>38328962</v>
       </c>
       <c r="BC16" t="n">
-        <v>3381000</v>
+        <v>38328962</v>
       </c>
       <c r="BD16" t="n">
         <v>0</v>
@@ -4315,45 +4315,45 @@
         <v>0</v>
       </c>
       <c r="BN16" t="n">
-        <v>0</v>
+        <v>2255167</v>
       </c>
       <c r="BO16" t="n">
-        <v>0</v>
+        <v>21276462</v>
       </c>
       <c r="BP16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BQ16" t="n">
         <v>0</v>
       </c>
       <c r="BR16" t="n">
-        <v>0</v>
+        <v>0.106</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>JAYAGROGN</t>
+          <t>ASAHISONG</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Jayant Agro-Organics Limited</t>
+          <t>ASAHI SONGWON COLORS LIMITED</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Fundamental Watch</t>
+          <t>Watchlist</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="G17" t="n">
         <v>21</v>
@@ -4362,28 +4362,28 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>234.84</v>
+        <v>402.75</v>
       </c>
       <c r="J17" t="n">
-        <v>234.4</v>
+        <v>338.1</v>
       </c>
       <c r="K17" t="n">
-        <v>0.2</v>
+        <v>19.1</v>
       </c>
       <c r="L17" t="n">
-        <v>67.13</v>
+        <v>66.73</v>
       </c>
       <c r="M17" t="n">
-        <v>0.3</v>
+        <v>0.34</v>
       </c>
       <c r="N17" t="n">
-        <v>2995877</v>
+        <v>3381000</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
       </c>
       <c r="P17" t="n">
-        <v>2995877</v>
+        <v>3381000</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -4397,124 +4397,124 @@
         <v>0</v>
       </c>
       <c r="T17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="V17" t="n">
-        <v>0.042</v>
+        <v>0.073</v>
       </c>
       <c r="W17" t="n">
-        <v>705</v>
+        <v>461</v>
       </c>
       <c r="X17" t="n">
-        <v>11.5</v>
+        <v>13.6</v>
       </c>
       <c r="Y17" t="n">
-        <v>-5</v>
+        <v>-8</v>
       </c>
       <c r="Z17" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="AA17" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="AB17" t="n">
-        <v>6.54</v>
+        <v>14.36</v>
       </c>
       <c r="AC17" t="n">
-        <v>14.8</v>
+        <v>9.94</v>
       </c>
       <c r="AD17" t="n">
-        <v>0.11</v>
+        <v>0.23</v>
       </c>
       <c r="AE17" t="b">
         <v>1</v>
       </c>
       <c r="AF17" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="AG17" t="n">
-        <v>227.7</v>
+        <v>359.64</v>
       </c>
       <c r="AH17" t="n">
-        <v>205.16</v>
+        <v>270.07</v>
       </c>
       <c r="AI17" t="n">
-        <v>40.7</v>
+        <v>101.1</v>
       </c>
       <c r="AJ17" t="n">
-        <v>234.4008293560754</v>
+        <v>338.1</v>
       </c>
       <c r="AK17" t="n">
-        <v>0.2</v>
+        <v>19.1</v>
       </c>
       <c r="AL17" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Aging</t>
         </is>
       </c>
       <c r="AM17" t="inlineStr">
         <is>
-          <t>Early Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AN17" t="inlineStr">
         <is>
-          <t>Early Accumulation</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AO17" t="inlineStr">
         <is>
-          <t>21-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="AP17" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="AQ17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AR17" t="n">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="AS17" t="n">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="AT17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AU17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AV17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AW17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AX17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AY17" t="n">
-        <v>1358248</v>
+        <v>0</v>
       </c>
       <c r="AZ17" t="n">
-        <v>2995877</v>
+        <v>0</v>
       </c>
       <c r="BA17" t="n">
-        <v>2995877</v>
+        <v>0</v>
       </c>
       <c r="BB17" t="n">
-        <v>2995877</v>
+        <v>3381000</v>
       </c>
       <c r="BC17" t="n">
-        <v>2995877</v>
+        <v>3381000</v>
       </c>
       <c r="BD17" t="n">
         <v>0</v>
@@ -4547,10 +4547,10 @@
         <v>0</v>
       </c>
       <c r="BN17" t="n">
-        <v>1358248</v>
+        <v>0</v>
       </c>
       <c r="BO17" t="n">
-        <v>2995877</v>
+        <v>0</v>
       </c>
       <c r="BP17" t="n">
         <v>1</v>
@@ -4559,18 +4559,18 @@
         <v>0</v>
       </c>
       <c r="BR17" t="n">
-        <v>0.4534</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>JAYAGROGN</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
+          <t>Jayant Agro-Organics Limited</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -4582,40 +4582,40 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F18" t="n">
         <v>12</v>
       </c>
       <c r="G18" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="H18" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>191.99</v>
+        <v>234.84</v>
       </c>
       <c r="J18" t="n">
-        <v>170.45</v>
+        <v>234.4</v>
       </c>
       <c r="K18" t="n">
-        <v>12.6</v>
+        <v>0.2</v>
       </c>
       <c r="L18" t="n">
-        <v>67.54000000000001</v>
+        <v>67.13</v>
       </c>
       <c r="M18" t="n">
-        <v>0.26</v>
+        <v>0.3</v>
       </c>
       <c r="N18" t="n">
-        <v>2560187</v>
+        <v>2995877</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>2560187</v>
+        <v>2995877</v>
       </c>
       <c r="Q18" t="n">
         <v>0</v>
@@ -4629,124 +4629,124 @@
         <v>0</v>
       </c>
       <c r="T18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
       <c r="V18" t="n">
-        <v>0.099</v>
+        <v>0.043</v>
       </c>
       <c r="W18" t="n">
-        <v>258</v>
+        <v>689</v>
       </c>
       <c r="X18" t="n">
-        <v>27.6</v>
+        <v>11.2</v>
       </c>
       <c r="Y18" t="n">
-        <v>24</v>
+        <v>-5</v>
       </c>
       <c r="Z18" t="n">
-        <v>1.87</v>
+        <v>32</v>
       </c>
       <c r="AA18" t="n">
-        <v>-31</v>
+        <v>1</v>
       </c>
       <c r="AB18" t="n">
-        <v>3.36</v>
+        <v>6.54</v>
       </c>
       <c r="AC18" t="n">
-        <v>4.96</v>
+        <v>14.8</v>
       </c>
       <c r="AD18" t="n">
-        <v>0</v>
+        <v>0.11</v>
       </c>
       <c r="AE18" t="b">
         <v>1</v>
       </c>
       <c r="AF18" t="n">
-        <v>2.97</v>
+        <v>9</v>
       </c>
       <c r="AG18" t="n">
-        <v>181.14</v>
+        <v>227.7</v>
       </c>
       <c r="AH18" t="n">
-        <v>163.73</v>
+        <v>205.16</v>
       </c>
       <c r="AI18" t="n">
-        <v>57.4</v>
+        <v>40.7</v>
       </c>
       <c r="AJ18" t="n">
-        <v>170.4518641810919</v>
+        <v>234.4008293560754</v>
       </c>
       <c r="AK18" t="n">
-        <v>12.6</v>
+        <v>0.2</v>
       </c>
       <c r="AL18" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AM18" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Early Accumulation</t>
         </is>
       </c>
       <c r="AN18" t="inlineStr">
         <is>
-          <t>Mature — Wait for Pullback</t>
+          <t>Early Accumulation</t>
         </is>
       </c>
       <c r="AO18" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>21-09-2026</t>
         </is>
       </c>
       <c r="AP18" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
       <c r="AQ18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AR18" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="AS18" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="AT18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AU18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AV18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AX18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AY18" t="n">
-        <v>0</v>
+        <v>1358248</v>
       </c>
       <c r="AZ18" t="n">
-        <v>0</v>
+        <v>2995877</v>
       </c>
       <c r="BA18" t="n">
-        <v>2560187</v>
+        <v>2995877</v>
       </c>
       <c r="BB18" t="n">
-        <v>2560187</v>
+        <v>2995877</v>
       </c>
       <c r="BC18" t="n">
-        <v>2560187</v>
+        <v>2995877</v>
       </c>
       <c r="BD18" t="n">
         <v>0</v>
@@ -4779,19 +4779,19 @@
         <v>0</v>
       </c>
       <c r="BN18" t="n">
-        <v>0</v>
+        <v>1358248</v>
       </c>
       <c r="BO18" t="n">
-        <v>2560187</v>
+        <v>2995877</v>
       </c>
       <c r="BP18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BQ18" t="n">
         <v>0</v>
       </c>
       <c r="BR18" t="n">
-        <v>0</v>
+        <v>0.4534</v>
       </c>
     </row>
     <row r="19">
@@ -4869,13 +4869,13 @@
         </is>
       </c>
       <c r="V19" t="n">
-        <v>2.86</v>
+        <v>2.844</v>
       </c>
       <c r="W19" t="n">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="X19" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="Y19" t="n">
         <v>30</v>
@@ -5095,13 +5095,13 @@
         </is>
       </c>
       <c r="V20" t="n">
-        <v>0.624</v>
+        <v>0.633</v>
       </c>
       <c r="W20" t="n">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="X20" t="n">
-        <v>1214</v>
+        <v>1196</v>
       </c>
       <c r="Y20" t="n">
         <v>-61</v>
@@ -5323,13 +5323,13 @@
         </is>
       </c>
       <c r="V21" t="n">
-        <v>0.265</v>
+        <v>0.267</v>
       </c>
       <c r="W21" t="n">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="X21" t="n">
-        <v>39.1</v>
+        <v>38.7</v>
       </c>
       <c r="Y21" t="n">
         <v>-44</v>
@@ -5555,13 +5555,13 @@
         </is>
       </c>
       <c r="V22" t="n">
-        <v>0.493</v>
+        <v>0.497</v>
       </c>
       <c r="W22" t="n">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="X22" t="n">
-        <v>37.6</v>
+        <v>37.3</v>
       </c>
       <c r="Y22" t="n">
         <v>21</v>
@@ -5790,10 +5790,10 @@
         <v>0.07099999999999999</v>
       </c>
       <c r="W23" t="n">
-        <v>800</v>
+        <v>796</v>
       </c>
       <c r="X23" t="n">
-        <v>20.2</v>
+        <v>20.1</v>
       </c>
       <c r="Y23" t="n">
         <v>19</v>
@@ -6017,10 +6017,10 @@
         </is>
       </c>
       <c r="V24" t="n">
-        <v>0.025</v>
+        <v>0.024</v>
       </c>
       <c r="W24" t="n">
-        <v>999</v>
+        <v>1010</v>
       </c>
       <c r="X24" t="inlineStr"/>
       <c r="Y24" t="n">
@@ -6250,10 +6250,10 @@
         <v>0.162</v>
       </c>
       <c r="W25" t="n">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="X25" t="n">
-        <v>57.3</v>
+        <v>57.2</v>
       </c>
       <c r="Y25" t="n">
         <v>3</v>
@@ -6271,7 +6271,7 @@
         <v>11.6</v>
       </c>
       <c r="AD25" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AE25" t="b">
         <v>1</v>
@@ -6479,13 +6479,13 @@
         </is>
       </c>
       <c r="V26" t="n">
-        <v>0.059</v>
+        <v>0.057</v>
       </c>
       <c r="W26" t="n">
-        <v>1874</v>
+        <v>1916</v>
       </c>
       <c r="X26" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="Y26" t="n">
         <v>20</v>
@@ -6714,10 +6714,10 @@
         <v>0.05</v>
       </c>
       <c r="W27" t="n">
-        <v>5246</v>
+        <v>5231</v>
       </c>
       <c r="X27" t="n">
-        <v>34.2</v>
+        <v>34.1</v>
       </c>
       <c r="Y27" t="n">
         <v>-25</v>
@@ -6943,13 +6943,13 @@
         </is>
       </c>
       <c r="V28" t="n">
-        <v>0.135</v>
+        <v>0.132</v>
       </c>
       <c r="W28" t="n">
-        <v>368</v>
+        <v>377</v>
       </c>
       <c r="X28" t="n">
-        <v>5.93</v>
+        <v>6.1</v>
       </c>
       <c r="Y28" t="n">
         <v>118</v>
@@ -7171,13 +7171,13 @@
         </is>
       </c>
       <c r="V29" t="n">
-        <v>0.858</v>
+        <v>0.866</v>
       </c>
       <c r="W29" t="n">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="X29" t="n">
-        <v>6.75</v>
+        <v>6.7</v>
       </c>
       <c r="Y29" t="n">
         <v>31</v>
@@ -7399,13 +7399,13 @@
         </is>
       </c>
       <c r="V30" t="n">
-        <v>0.641</v>
+        <v>0.644</v>
       </c>
       <c r="W30" t="n">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="X30" t="n">
-        <v>11.3</v>
+        <v>11.2</v>
       </c>
       <c r="Y30" t="n">
         <v>19</v>
@@ -7631,13 +7631,13 @@
         </is>
       </c>
       <c r="V31" t="n">
-        <v>0.038</v>
+        <v>0.039</v>
       </c>
       <c r="W31" t="n">
-        <v>3490</v>
+        <v>3423</v>
       </c>
       <c r="X31" t="n">
-        <v>20.7</v>
+        <v>20.3</v>
       </c>
       <c r="Y31" t="n">
         <v>-4</v>
@@ -7866,10 +7866,10 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W32" t="n">
-        <v>53444</v>
+        <v>53455</v>
       </c>
       <c r="X32" t="n">
-        <v>45.3</v>
+        <v>45.2</v>
       </c>
       <c r="Y32" t="n">
         <v>5</v>
@@ -8095,13 +8095,13 @@
         </is>
       </c>
       <c r="V33" t="n">
-        <v>0.308</v>
+        <v>0.315</v>
       </c>
       <c r="W33" t="n">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="X33" t="n">
-        <v>24.3</v>
+        <v>23.8</v>
       </c>
       <c r="Y33" t="n">
         <v>12</v>
@@ -8330,10 +8330,10 @@
         <v>0</v>
       </c>
       <c r="W34" t="n">
-        <v>3748</v>
+        <v>3527</v>
       </c>
       <c r="X34" t="n">
-        <v>84.40000000000001</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="Y34" t="n">
         <v>42</v>
@@ -8559,13 +8559,13 @@
         </is>
       </c>
       <c r="V35" t="n">
-        <v>0.02</v>
+        <v>0.021</v>
       </c>
       <c r="W35" t="n">
-        <v>9589</v>
+        <v>9522</v>
       </c>
       <c r="X35" t="n">
-        <v>12.7</v>
+        <v>12.6</v>
       </c>
       <c r="Y35" t="n">
         <v>-12</v>
@@ -9020,10 +9020,10 @@
         <v>0.008</v>
       </c>
       <c r="W37" t="n">
-        <v>5427</v>
+        <v>5218</v>
       </c>
       <c r="X37" t="n">
-        <v>9.17</v>
+        <v>8.82</v>
       </c>
       <c r="Y37" t="n">
         <v>43</v>
@@ -9252,7 +9252,7 @@
         <v>0.217</v>
       </c>
       <c r="W38" t="n">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="X38" t="n">
         <v>14.2</v>
@@ -9481,13 +9481,13 @@
         </is>
       </c>
       <c r="V39" t="n">
-        <v>0.208</v>
+        <v>0.211</v>
       </c>
       <c r="W39" t="n">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="X39" t="n">
-        <v>25.7</v>
+        <v>25.3</v>
       </c>
       <c r="Y39" t="n">
         <v>21</v>
@@ -9713,13 +9713,13 @@
         </is>
       </c>
       <c r="V40" t="n">
-        <v>0.212</v>
+        <v>0.214</v>
       </c>
       <c r="W40" t="n">
-        <v>966</v>
+        <v>957</v>
       </c>
       <c r="X40" t="n">
-        <v>26.3</v>
+        <v>26.1</v>
       </c>
       <c r="Y40" t="n">
         <v>9</v>
@@ -10180,10 +10180,10 @@
         <v>0.074</v>
       </c>
       <c r="W42" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="X42" t="n">
-        <v>13.2</v>
+        <v>13.3</v>
       </c>
       <c r="Y42" t="n">
         <v>185</v>
@@ -10410,7 +10410,7 @@
         <v>0</v>
       </c>
       <c r="W43" t="n">
-        <v>8983</v>
+        <v>8932</v>
       </c>
       <c r="X43" t="n">
         <v>15.2</v>
@@ -10639,13 +10639,13 @@
         </is>
       </c>
       <c r="V44" t="n">
-        <v>0.6870000000000001</v>
+        <v>0.674</v>
       </c>
       <c r="W44" t="n">
-        <v>3789</v>
+        <v>3864</v>
       </c>
       <c r="X44" t="n">
-        <v>26.5</v>
+        <v>27</v>
       </c>
       <c r="Y44" t="n">
         <v>2</v>
@@ -10871,13 +10871,13 @@
         </is>
       </c>
       <c r="V45" t="n">
-        <v>0.224</v>
+        <v>0.227</v>
       </c>
       <c r="W45" t="n">
-        <v>1785</v>
+        <v>1758</v>
       </c>
       <c r="X45" t="n">
-        <v>18.9</v>
+        <v>18.6</v>
       </c>
       <c r="Y45" t="n">
         <v>-3</v>
@@ -11106,10 +11106,10 @@
         <v>0</v>
       </c>
       <c r="W46" t="n">
-        <v>118820</v>
+        <v>117300</v>
       </c>
       <c r="X46" t="n">
-        <v>34.2</v>
+        <v>33.8</v>
       </c>
       <c r="Y46" t="n">
         <v>18</v>
@@ -11335,13 +11335,13 @@
         </is>
       </c>
       <c r="V47" t="n">
-        <v>0.356</v>
+        <v>0.36</v>
       </c>
       <c r="W47" t="n">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="X47" t="n">
-        <v>97.2</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="Y47" t="n">
         <v>246</v>
@@ -11567,13 +11567,13 @@
         </is>
       </c>
       <c r="V48" t="n">
-        <v>0.043</v>
+        <v>0.044</v>
       </c>
       <c r="W48" t="n">
-        <v>1613</v>
+        <v>1589</v>
       </c>
       <c r="X48" t="n">
-        <v>21.1</v>
+        <v>20.8</v>
       </c>
       <c r="Y48" t="n">
         <v>10</v>
@@ -11802,10 +11802,10 @@
         <v>0.082</v>
       </c>
       <c r="W49" t="n">
-        <v>1671</v>
+        <v>1659</v>
       </c>
       <c r="X49" t="n">
-        <v>30.2</v>
+        <v>30</v>
       </c>
       <c r="Y49" t="n">
         <v>39</v>
@@ -12486,140 +12486,140 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>STEL</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>STEL HOLDINGS LIMITED</t>
+          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>619.3</v>
+        <v>191.99</v>
       </c>
       <c r="D15" t="n">
-        <v>636.71</v>
+        <v>170.45</v>
       </c>
       <c r="E15" t="n">
-        <v>-2.7</v>
+        <v>12.6</v>
       </c>
       <c r="F15" t="n">
-        <v>64.68000000000001</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>4.12</v>
+        <v>0.26</v>
       </c>
       <c r="H15" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ASAHISONG</t>
+          <t>STEL</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ASAHI SONGWON COLORS LIMITED</t>
+          <t>STEL HOLDINGS LIMITED</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>402.75</v>
+        <v>619.3</v>
       </c>
       <c r="D16" t="n">
-        <v>338.1</v>
+        <v>636.71</v>
       </c>
       <c r="E16" t="n">
-        <v>19.1</v>
+        <v>-2.7</v>
       </c>
       <c r="F16" t="n">
-        <v>66.73</v>
+        <v>64.68000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>0.34</v>
+        <v>4.12</v>
       </c>
       <c r="H16" t="n">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>JAYAGROGN</t>
+          <t>ASAHISONG</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Jayant Agro-Organics Limited</t>
+          <t>ASAHI SONGWON COLORS LIMITED</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>234.84</v>
+        <v>402.75</v>
       </c>
       <c r="D17" t="n">
-        <v>234.4</v>
+        <v>338.1</v>
       </c>
       <c r="E17" t="n">
-        <v>0.2</v>
+        <v>19.1</v>
       </c>
       <c r="F17" t="n">
-        <v>67.13</v>
+        <v>66.73</v>
       </c>
       <c r="G17" t="n">
-        <v>0.3</v>
+        <v>0.34</v>
       </c>
       <c r="H17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>JAYAGROGN</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
+          <t>Jayant Agro-Organics Limited</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>191.99</v>
+        <v>234.84</v>
       </c>
       <c r="D18" t="n">
-        <v>170.45</v>
+        <v>234.4</v>
       </c>
       <c r="E18" t="n">
-        <v>12.6</v>
+        <v>0.2</v>
       </c>
       <c r="F18" t="n">
-        <v>67.54000000000001</v>
+        <v>67.13</v>
       </c>
       <c r="G18" t="n">
-        <v>0.26</v>
+        <v>0.3</v>
       </c>
       <c r="H18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
     </row>
@@ -13811,7 +13811,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -13831,7 +13831,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>